<commit_message>
Actualizar las slides y DEF-022 con el fix verificado en producción
- Slide de defectos: 16 abiertos (se suma DEF-021, Media), 6 corregidos
  (se suma DEF-022, Crítica) y 6 nuevos, igual que 04-reportes-de-defectos.
- DEF-022: las migraciones ya se aplicaron en producción con supabase db
  push y el flujo se verificó allí; se saca el "falta aplicar".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-1/04-reportes-de-defectos.xlsx
+++ b/entrega-1/04-reportes-de-defectos.xlsx
@@ -1349,7 +1349,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Cerrado · corregido en #176 el 2026-09-29; verificado en local (falta aplicar las migraciones en producción)</t>
+          <t>Cerrado · corregido en #176 el 2026-09-29; migraciones aplicadas y verificado en producción el 2026-09-29</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -3736,7 +3736,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="375" customHeight="1">
+    <row r="22" ht="390" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
@@ -3745,14 +3745,14 @@
       <c r="B22" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-022
-- Estado: Cerrado · corregido en #176 el 2026-09-29; verificado en local (falta aplicar las migraciones en producción)
+- Estado: Cerrado · corregido en #176 el 2026-09-29; migraciones aplicadas y verificado en producción el 2026-09-29
 - Issue de GitHub: #175
 - Caso de prueba: — (no había caso; se agregaron los tests de regresión de e2e/setup.spec.ts)
 - Encontrado en: uso en producción después del merge de #173 (US-68), fuera del catálogo escrito.
 - Reportó: Uso en producción (usuario con cuenta previa), analizado con Claude Code, equipo Biyu
 - Evidencia: Tests de regresión en rojo antes de la corrección: e2e/setup.spec.ts (fallan "si guardar el setup falla", "si leer el estado falla" y "cuenta sin fila") y e2e/smoke.spec.ts (esperaba /register después del signup). Después de #176: e2e 28/28 en Chromium y WebKit, pgTAP 175/175, Vitest 246/246.
 - Corrección: PR #176 (ADR-025 §6): la fila pendiente la crea la base al registrarse, y el guard deja entrar a la app si leer o guardar falla.
-- No saltó ninguna alarma porque ningún test cubría cuentas previas ni fallas al guardar, y la prueba de humo, que sí fallaba, no corre en la CI. Corrección (ADR-025 §6): trigger que crea la fila pendiente al registrarse (sin fila = cuenta anterior) y el guard falla abierto. Pendiente: correr supabase db push en producción.</t>
+- No saltó ninguna alarma porque ningún test cubría cuentas previas ni fallas al guardar, y la prueba de humo, que sí fallaba, no corre en la CI. Corrección (ADR-025 §6): trigger que crea la fila pendiente al registrarse (sin fila = cuenta anterior) y el guard falla abierto. Las migraciones se aplicaron en producción con supabase db push y el flujo se verificó allí.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Detallar botón por botón los pasos de reproducción de los 22 defectos
Los pasos daban por sabido cómo llegar al defecto ("Crear un gasto en
Entretenimiento", "Archivar desde /settings", "POST … con JWT válido").
El template de defectos no tiene campo de pre-requisitos, así que ahora
cada reproducción arranca desde cero: iniciar sesión, preparar los datos
con los botones y campos reales de la pantalla, y recién después lo que
dispara el defecto.

- Las reproducciones por API dicen cómo sacar el token y los ids, y qué
  cuerpo mandar.
- Los defectos ya corregidos (DEF-001 a 004, 017 y 022) aclaran en qué
  versión ocurrían.
- Solo cambian los pasos (44 -> 119): título, descripción, esperado,
  obtenido, severidad, estado y evidencia quedan igual.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entrega-1/04-reportes-de-defectos.xlsx
+++ b/entrega-1/04-reportes-de-defectos.xlsx
@@ -1403,7 +1403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -1434,7 +1434,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -1442,103 +1442,138 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Con una cuenta credit_card que ya tiene compras en cuotas (2, 3, 12).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- PATCH /rest/v1/accounts?id=eq.&lt;esa cuenta&gt; con {"type":"cash"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+          <t>2- Tocar el engranaje "Ajustes" arriba a la derecha (en computadora, "Ajustes" en el menú lateral). En "Cuentas", escribir "Visa BBVA" en "Nueva cuenta", elegir "Tarjeta de crédito" en "Tipo" y tocar "Crear cuenta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="105" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Registrar tres compras en cuotas con esa cuenta. En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar". Después: escribir 12000 en el monto, tocar "Siguiente", tocar el chip "Otros", en "Cuenta" tocar "Visa BBVA", en "Cuotas" tocar "2", tocar "Guardar gasto" (aparece "Gasto guardado"). Repetir con "3" y con "12" en "Cuotas".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Obtener el token de sesión del usuario (en la consola del navegador, con la app abierta: la clave "sb-…-auth-token" de localStorage, campo access_token) y la anon key del proyecto. Las llamadas de los pasos siguientes llevan los encabezados "apikey: &lt;anon key&gt;" y "Authorization: Bearer &lt;token&gt;".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Obtener el id de "Visa BBVA": GET /rest/v1/accounts?select=id,name&amp;name=eq.Visa BBVA. La pantalla no permite editar cuentas (DEF-011), por eso el cambio se hace por API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Llamar a PATCH /rest/v1/accounts?id=eq.&lt;id de Visa BBVA&gt; con el cuerpo {"type": "cash"}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>7- Leer la respuesta y, en la base local, consultar las compras de esa cuenta: select installments_count from transactions where account_id = '&lt;id&gt;' and deleted_at is null.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>I6 ("installments_count &gt; 1 solo si la cuenta es credit_card") debería impedir este estado, o al menos advertirlo — el trigger actual (check_installments_rule) solo corre sobre transactions, nunca se dispara al editar accounts</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Actual Behavior</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>200, el tipo cambia. Las transacciones existentes quedan con installments_count &gt; 1 sobre una cuenta ahora cash</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Incidence / Severity / Probability of reproduction</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Severidad Media - Quedan compras en cuotas sobre una cuenta que ya no es tarjeta de crédito: se rompe la invariante I6 después de creada la transacción.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>200, el tipo cambia. Las transacciones existentes quedan con installments_count &gt; 1 sobre una cuenta ahora cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Severidad Media - Quedan compras en cuotas sobre una cuenta que ya no es tarjeta de crédito: se rompe la invariante I6 después de creada la transacción.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>US-45 · Crear cuentas indicando su tipo. Criterio: "El tipo determina si admite cuotas (I6)."</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright) y consulta directa a la base</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="195" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="26" ht="195" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-009
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -1561,7 +1596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -1592,7 +1627,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -1600,103 +1635,131 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Archivar las 8 categorías sembradas de un usuario (desde la UI o la API).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Abrir /register con ese usuario</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+          <t>2- Tocar el engranaje "Ajustes" arriba a la derecha (en computadora, "Ajustes" en el menú lateral).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- En "Categorías", tocar el botón de archivar ("Archivar …") a la derecha de cada una de las 8 categorías sembradas (Comida y supermercado, Transporte, Servicios, Entretenimiento, Salud, Educación, Indumentaria, Otros), una por una, hasta que la lista quede vacía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Escribir cualquier monto y tocar "Siguiente": mirar la grilla de categorías.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Volver a Ajustes y mirar la lista "Categorías". En la base local, contar las categorías del usuario: select count(*), count(*) filter (where archived_at is null) from categories where user_id = '&lt;id&gt;'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Respetar la decisión del usuario de no tener categorías activas; ADR-014 pensó la red de contención de /register solo para un usuario que nunca se sembró, no para uno que archivó todo a propósito</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Aparecen 8 categorías activas nuevas (recién creadas), además de las 8 archivadas — 16 filas en total</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Severidad Media - El usuario que archivó todas sus categorías las vuelve a ver aparecer duplicadas (8 nuevas además de las archivadas).</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="B13" s="7" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>US-43 · Set inicial de categorías y cuentas. Criterio: "La siembra es por usuario y no se repite si ya existe (ADR-014)."</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="180" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="25" ht="180" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-010
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -1719,7 +1782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -1750,7 +1813,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -1758,96 +1821,117 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Abrir /settings, sección "Cuentas"</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- Tocar el engranaje "Ajustes" arriba a la derecha (en computadora, "Ajustes" en el menú lateral).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Mirar la sección "Categorías": cada fila tiene un lápiz ("Editar …") y un botón de archivar ("Archivar …").</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Mirar la sección "Cuentas": buscar en cada fila un botón para editar el nombre o el tipo, o para archivar la cuenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>FR-05: "el usuario puede crear, editar y dar de baja **sus propias categorías y medios de pago**" — solo la mitad (categorías) está implementada</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Cada fila muestra solo nombre y tipo, sin acciones. Las categorías sí tienen "Editar" y "Archivar" (settings-categories-edit/-archive); las cuentas no tienen equivalente</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Severidad Media - Una cuenta creada con un error de nombre o de tipo no se puede corregir ni sacar de la lista.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>US-45 · Crear cuentas indicando su tipo. Criterio: "ABM de cuentas con tipo (credit_card, débito, efectivo, etc.)." Solo existe el alta.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="165" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="23" ht="165" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-011
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -1870,7 +1954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -1901,7 +1985,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -1909,96 +1993,131 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- En /register, monto 1000000000000 (excede numeric(14,2)), completar el resto y Guardar</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Escribir 1000000000000 en el monto (un billón: supera el máximo de numeric(14,2)). "Siguiente" queda habilitado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Tocar "Siguiente" y después el chip "Otros".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- En "Cuenta", tocar "Tarjeta de crédito" y en "Cuotas" tocar "2". Leer la previsualización ("2 cuotas de $500.000.000.000,00").</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Tocar "Guardar gasto" y leer el aviso que aparece arriba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Validación de cliente que rechace el monto antes de enviarlo, con un mensaje en español ("El monto máximo permitido es…")</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Actual Behavior</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>La previsualización de cuotas lo muestra normal ("2 cuotas de $500.000.000.000,00"). Al guardar: toast "No se pudo guardar / numeric field overflow" (mensaje técnico en inglés)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Incidence / Severity / Probability of reproduction</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Severidad Baja - Un monto fuera de rango pasa la validación de la pantalla y falla recién al guardar, con un mensaje técnico en inglés.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>La previsualización de cuotas lo muestra normal ("2 cuotas de $500.000.000.000,00"). Al guardar: toast "No se pudo guardar / numeric field overflow" (mensaje técnico en inglés)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Severidad Baja - Un monto fuera de rango pasa la validación de la pantalla y falla recién al guardar, con un mensaje técnico en inglés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>US-11 · No se puede guardar monto cero o negativo. Los criterios cubren monto vacío, 0 o negativo; el límite superior (numeric(14,2)) no tiene criterio escrito.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="165" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="25" ht="165" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-012
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -2021,7 +2140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -2052,7 +2171,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -2060,96 +2179,131 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- En /register: moneda USD, monto 0,01, TC 0,01, cuenta no crediticia (para que no haya selector de cuotas visible)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Tocar "US$". Escribir 0,01 en el monto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- En "Tipo de cambio (ARS por US$)", borrar el valor y escribir 0,01. Tocar "Siguiente".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Tocar el chip "Otros". En "Cuenta", tocar "Efectivo" (una cuenta que no es de crédito, así no aparece el selector de cuotas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Mirar el botón "Guardar gasto" y buscar en la pantalla algún mensaje que explique por qué no se puede guardar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Un mensaje visible que explique por qué no se puede guardar, sin importar si el selector de cuotas está oculto</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="14" ht="75" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>El botón Guardar queda deshabilitado, sin ningún texto de error visible. El motivo real ("Con ese monto, cada cuota daría menos de 0,01") lo genera validateTransactionDraft pero lo asigna al campo de cuotas, que no se renderiza con esa cuenta</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Severidad Baja - El botón Guardar queda deshabilitado sin que la pantalla diga por qué.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>US-19 · Registrar un gasto en USD sin convertir a mano. Aplica el criterio de US-11: "el botón queda deshabilitado y el campo dice por qué".</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="195" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="25" ht="195" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-013
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -2172,7 +2326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -2203,7 +2357,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -2211,96 +2365,117 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Abrir /dashboard?period=0000-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- Escribir en la barra del navegador la dirección de la app seguida de /dashboard?period=0000-01 y dar Enter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Leer el mensaje que muestra el Resumen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Para comparar, repetir con /dashboard?period=2026-13 y /dashboard?period=fecha-invalida: esos vuelven al mes actual sin error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Igual que otros períodos inválidos (2026-13, fecha-invalida, &lt;script&gt;, 9999-12+"→"): volver silenciosamente al mes actual, sin error visible</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>"No se pudo cargar el resumen: date/time field value out of range: …" (mensaje técnico de Postgres, en inglés)</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Severidad Baja - Un período inválido en la URL muestra un error técnico de la base, en inglés.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>US-26 · Cambiar de mes con un selector. Criterio: "El período vive en la URL (?period=AAAA-MM) y es enlazable (C11)." No hay criterio para un período inválido.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="165" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="23" ht="165" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-014
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -2323,7 +2498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -2354,7 +2529,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -2362,96 +2537,131 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Recorrer los elementos interactivos de /settings</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- Tocar el engranaje "Ajustes" arriba a la derecha (en computadora, "Ajustes" en el menú lateral).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Abrir las herramientas de desarrollo (F12), pestaña "Elements" (o "Inspector").</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- En la sección "Categorías", hacer clic derecho sobre un círculo de color de la paleta de "Nueva categoría" y elegir "Inspeccionar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- En el HTML del botón (aria-label con el color, por ejemplo "#f97316"), buscar el atributo data-testid. Repetir con los demás colores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Inspeccionar también los botones de lápiz y de archivar de dos categorías distintas y comparar sus data-testid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>"Todo elemento interactivo lleva data-testid" (07-plan-de-testing.md §2); "un elemento interactivo sin data-testid es un defecto de testeabilidad"</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Los 10 botones de color (aria-label="#f97316" … "#0ea5e9") tienen data-testid = null. Además settings-categories-edit/-archive se repiten idénticos en cada fila de categoría (sin distinguir cuál)</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Severidad Baja - No afecta al usuario. Impide automatizar la elección de color en V3.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Transversal, sin historia propia. Regla del plan de testing (07-plan-de-testing.md §2): todo elemento interactivo lleva data-testid.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="150" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="25" ht="150" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-015
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -2474,7 +2684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -2505,7 +2715,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -2513,96 +2723,138 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Con sesión válida, POST /rest/v1/debts con un transaction_id propio válido y un monto que cumple I7 (menor o igual al gasto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+          <t>1- Afecta a las deudas, que son de V2 y no tienen pantalla: se reproduce por API, contra el stack local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar". Después: escribir 1000 en el monto, tocar "Siguiente", tocar el chip "Otros", en "Cuenta" tocar "Efectivo", tocar "Guardar gasto" (aparece "Gasto guardado").</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Obtener el token de sesión del usuario (en la consola del navegador, con la app abierta: la clave "sb-…-auth-token" de localStorage, campo access_token) y la anon key del proyecto. Las llamadas de los pasos siguientes llevan los encabezados "apikey: &lt;anon key&gt;" y "Authorization: Bearer &lt;token&gt;".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Obtener el id de ese gasto: GET /rest/v1/transactions?select=id,amount&amp;order=created_at.desc&amp;limit=1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Llamar a POST /rest/v1/debts con el cuerpo {"transaction_id": "&lt;id del gasto&gt;", "person": "Sofi", "amount": "500", "currency": "ARS", "direction": "owed_to_me", "incurred_on": "&lt;fecha de hoy&gt;"}. El monto (500) es menor que el gasto (1000), así que cumple I7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>7- Leer el código y el mensaje de la respuesta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Aceptar una deuda válida; rechazar solo las que violan I7 con un mensaje de I7 — hoy rechaza **todas**, válidas o no</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="15" ht="75" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>42501 "permission denied for table transactions", con hint "GRANT UPDATE ON public.transactions". El trigger check_debt_rule hace select … for update sobre transactions sin security definer, así que corre con los permisos del cliente (que no tiene UPDATE sobre esa tabla, C4)</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Severidad Media - Latente: las deudas no son de V1, pero cuando se implementen no se va a poder crear ninguna deuda vinculada.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Sin historia de V1. Afecta a la invariante I7 de las deudas (V2), cuyo trigger ya está en el schema.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>No aplica: consulta directa a la base</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="210" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="26" ht="210" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-016
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -2620,6 +2872,380 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>[DEF-017] Después de crear la cuenta no aparece la configuración inicial (US-68 sin implementar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>La historia US-68 entra en el alcance de la Entrega 1 pero no tiene implementación: no hay ruta, pantalla ni componentes de setup en src/. El issue #159 sigue abierto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>1- Versión donde ocurría: main 44f1519, antes de #173 (US-68 sin implementar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- Abrir la app sin sesión. En /login, tocar "Crear una cuenta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Escribir un email nuevo en "Email", Clave123! en "Contraseña" y Clave123! en "Confirmar contraseña". Los cinco criterios se marcan con ✓.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Tocar "Crear cuenta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Observar la pantalla que se abre y la URL: si aparece la configuración inicial ("¿Para qué vas a usar Biyu?") o se va directo a Registrar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>US-68: después de crear la cuenta se muestra el setup (para qué la usás, categorías, cuentas y primer gasto), con elementos data-testid de prefijo setup-.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>La app va directo a /register. No hay ningún elemento con data-testid que empiece con setup-.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Severidad Alta - La configuración inicial comprometida para la Entrega 1 no existía: sus 5 casos no podían pasar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>100 % antes de la corrección. No se reproduce desde el 2026-09-29.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>US-68 · Configuración inicial al crear la cuenta. Criterio: "Después de crear la cuenta se muestra el setup, y no vuelve a aparecer una vez que se completó o se salteó."</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright), emulando un celular de 390×844</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Local: Vite http://localhost:5180 + Supabase local, main 44f1519, Chromium 390×844, 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="240" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-017
+- Estado: Cerrado · corregido en #173; CP-CFG-011 a CP-CFG-015 pasan en el re-test del 2026-09-29
+- Issue de GitHub: #165
+- Caso de prueba: CP-CFG-011 (bloquea CP-CFG-012 a CP-CFG-015)
+- Encontrado en: Ejecución de la Entrega 1, caso CP-CFG-011
+- Reportó: Ejecución de la Entrega 1 (runner Playwright, Claude Code), supervisada por Joaquin Nuñez
+- Evidencia: evidencia/CP-CFG-011-sin-setup.jpg
+- Corrección: PR #173: implementación de US-68 (ADR-025). Re-test del 2026-09-29: CP-CFG-011 a CP-CFG-015 PASSED.
+- Es una historia sin implementar más que un error de código. Se reporta como defecto porque la historia está comprometida para esta versión y sus 5 casos no pueden pasar. Los casos CP-CFG-012 a CP-CFG-015 quedan BLOCKED por este defecto.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31.83" customWidth="1" min="1" max="1"/>
+    <col width="63.66" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>[DEF-018] El registro acepta un tipo de cambio con más de 4 decimales y la base lo redondea sin avisar</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Description / Overview</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>En Ajustes el tipo de cambio de referencia se valida a 4 decimales ("Usá hasta 4 decimales"), pero en el formulario de registro no: se puede guardar un TC con 5 decimales y la base lo redondea en silencio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Reproduction Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Tocar "US$". Escribir 100 en el monto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- En "Tipo de cambio (ARS por US$)", borrar el valor y escribir 1250,55555 (5 decimales). Mirar si aparece algún aviso y el equivalente "≈ $…" que muestra el campo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Tocar "Siguiente", tocar el chip "Otros", en "Cuenta" tocar "Efectivo" y tocar "Guardar gasto". Aparece "Gasto guardado".</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- En la base local, consultar la transacción guardada: select fx_rate, amount_ars from transactions order by created_at desc limit 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>7- Para comparar: en Ajustes → "Tipo de cambio de referencia", escribir 1250,55555 en "ARS por USD" y tocar "Guardar tipo de cambio": ahí sí se rechaza con "Usá hasta 4 decimales".</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Misma validación que en Ajustes: rechazar más de 4 decimales con un mensaje (C6: el cliente anticipa lo que la base va a hacer), o guardar exactamente lo que se mostró.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Se guarda sin aviso con fx_rate 1250.5556 y amount_ars 125055.56. El equivalente en pesos que mostraba el formulario se calculó con el valor sin redondear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Incidence / Severity / Probability of reproduction</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Severidad Baja - El tipo de cambio guardado no es el que escribió el usuario: la base lo redondea a 4 decimales sin avisar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>100 % (se reprodujo en la ejecución del 2026-09-28).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Story and Acceptance Criteria affected</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>US-21 · Pisar el tipo de cambio sugerido en una transacción. Criterio: "El TC ingresado a mano pisa al de referencia solo para esa transacción." Se guarda un valor distinto del ingresado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Chromium (Playwright), emulando un celular de 390×844</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Local: Vite http://localhost:5180 + Supabase local, main 44f1519, Chromium 390×844, 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="165" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>- Defect ID: DEF-018
+- Estado: Abierto · nuevo en la Entrega 1
+- Issue de GitHub: sin issue
+- Caso de prueba: — (exploración, relacionado con CP-CUO-010 y CP-CFG-010)
+- Encontrado en: Exploración negativa y de borde de la Entrega 1 (EXP-01)
+- Reportó: Ejecución de la Entrega 1 (exploración de bordes EXP-01)
+- Evidencia: Consulta a la base: fx_rate|amount_ars = 1250.5556|125055.56 (resultados.json, EXP-01).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2640,11 +3266,11 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>[DEF-017] Después de crear la cuenta no aparece la configuración inicial (US-68 sin implementar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="45" customHeight="1">
+          <t>[DEF-001] Ruta inexistente muestra el error crudo del router, sin salida a la app</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Description / Overview</t>
@@ -2652,11 +3278,11 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>La historia US-68 entra en el alcance de la Entrega 1 pero no tiene implementación: no hay ruta, pantalla ni componentes de setup en src/. El issue #159 sigue abierto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
+          <t>Ruta inexistente muestra el error crudo del router, sin salida a la app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -2664,25 +3290,25 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Ir a /signup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>1- Versión donde ocurría: producción antes de #163. Se reproduce con o sin sesión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Crear una cuenta con un email nuevo y la contraseña Clave123! repetida en "Confirmar contraseña".</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>2- Abrir el navegador (Chromium) y escribir en la barra de direcciones https://biyu-rust.vercel.app/no-existe-esta-ruta. Dar Enter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>3- Observar la pantalla que se abre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
+          <t>3- Observar la pantalla que se abre: el texto, si aparece el encabezado de Biyu y si hay algún botón o link para volver a la app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
@@ -2690,11 +3316,11 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>US-68: después de crear la cuenta se muestra el setup (para qué la usás, categorías, cuentas y primer gasto), con elementos data-testid de prefijo setup-.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+          <t>Una pantalla de "no encontrado" propia en español con un camino de vuelta a la app, o redirección a /</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
@@ -2702,7 +3328,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>La app va directo a /register. No hay ningún elemento con data-testid que empiece con setup-.</t>
+          <t>El body muestra textualmente "Unexpected Application Error!\n404 Not Found" — la pantalla de error por defecto de React Router. Sin header de Biyu, sin link a /register o /login, sin redirección</t>
         </is>
       </c>
     </row>
@@ -2714,14 +3340,14 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Severidad Alta - La configuración inicial comprometida para la Entrega 1 no existía: sus 5 casos no podían pasar.</t>
+          <t>Severidad Media - Una URL mal escrita deja al usuario en una pantalla de error en inglés, sin forma de volver a la app.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>100 % antes de la corrección. No se reproduce desde el 2026-09-29.</t>
+          <t>100 % antes de la corrección. No se reproduce desde el 2026-09-28.</t>
         </is>
       </c>
     </row>
@@ -2733,7 +3359,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>US-68 · Configuración inicial al crear la cuenta. Criterio: "Después de crear la cuenta se muestra el setup, y no vuelve a aparecer una vez que se completó o se salteó."</t>
+          <t>US-48 · La app pide login. Ningún criterio escrito cubre las rutas inexistentes: se detectó por ataque libre, fuera de los criterios.</t>
         </is>
       </c>
     </row>
@@ -2745,7 +3371,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Chromium (Playwright), emulando un celular de 390×844</t>
+          <t>Google Chrome (Chromium) en Windows 11</t>
         </is>
       </c>
     </row>
@@ -2757,335 +3383,17 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Local: Vite http://localhost:5180 + Supabase local, main 44f1519, Chromium 390×844, 2026-09-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="240" customHeight="1">
+          <t>Producción https://biyu-rust.vercel.app, navegador Chromium, Windows 11, 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="225" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>- Defect ID: DEF-017
-- Estado: Cerrado · corregido en #173; CP-CFG-011 a CP-CFG-015 pasan en el re-test del 2026-09-29
-- Issue de GitHub: #165
-- Caso de prueba: CP-CFG-011 (bloquea CP-CFG-012 a CP-CFG-015)
-- Encontrado en: Ejecución de la Entrega 1, caso CP-CFG-011
-- Reportó: Ejecución de la Entrega 1 (runner Playwright, Claude Code), supervisada por Joaquin Nuñez
-- Evidencia: evidencia/CP-CFG-011-sin-setup.jpg
-- Corrección: PR #173: implementación de US-68 (ADR-025). Re-test del 2026-09-29: CP-CFG-011 a CP-CFG-015 PASSED.
-- Es una historia sin implementar más que un error de código. Se reporta como defecto porque la historia está comprometida para esta versión y sus 5 casos no pueden pasar. Los casos CP-CFG-012 a CP-CFG-015 quedan BLOCKED por este defecto.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="31.83" customWidth="1" min="1" max="1"/>
-    <col width="63.66" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>[DEF-018] El registro acepta un tipo de cambio con más de 4 decimales y la base lo redondea sin avisar</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Description / Overview</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>En Ajustes el tipo de cambio de referencia se valida a 4 decimales ("Usá hasta 4 decimales"), pero en el formulario de registro no: se puede guardar un TC con 5 decimales y la base lo redondea en silencio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Reproduction Steps</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>1- Abrir /register, cargar USD 100 y escribir 1250,55555 como tipo de cambio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>2- Completar categoría y cuenta y guardar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>3- Consultar la transacción guardada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Expected Behavior</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Misma validación que en Ajustes: rechazar más de 4 decimales con un mensaje (C6: el cliente anticipa lo que la base va a hacer), o guardar exactamente lo que se mostró.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Actual Behavior</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Se guarda sin aviso con fx_rate 1250.5556 y amount_ars 125055.56. El equivalente en pesos que mostraba el formulario se calculó con el valor sin redondear.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Incidence / Severity / Probability of reproduction</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Severidad Baja - El tipo de cambio guardado no es el que escribió el usuario: la base lo redondea a 4 decimales sin avisar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>100 % (se reprodujo en la ejecución del 2026-09-28).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Story and Acceptance Criteria affected</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>US-21 · Pisar el tipo de cambio sugerido en una transacción. Criterio: "El TC ingresado a mano pisa al de referencia solo para esa transacción." Se guarda un valor distinto del ingresado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Browsers tested</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Chromium (Playwright), emulando un celular de 390×844</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Environment</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Local: Vite http://localhost:5180 + Supabase local, main 44f1519, Chromium 390×844, 2026-09-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="165" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>- Defect ID: DEF-018
-- Estado: Abierto · nuevo en la Entrega 1
-- Issue de GitHub: sin issue
-- Caso de prueba: — (exploración, relacionado con CP-CUO-010 y CP-CFG-010)
-- Encontrado en: Exploración negativa y de borde de la Entrega 1 (EXP-01)
-- Reportó: Ejecución de la Entrega 1 (exploración de bordes EXP-01)
-- Evidencia: Consulta a la base: fx_rate|amount_ars = 1250.5556|125055.56 (resultados.json, EXP-01).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="31.83" customWidth="1" min="1" max="1"/>
-    <col width="63.66" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>[DEF-001] Ruta inexistente muestra el error crudo del router, sin salida a la app</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Description / Overview</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Ruta inexistente muestra el error crudo del router, sin salida a la app.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Reproduction Steps</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>1- Sin sesión (o con sesión), abrir https://biyu-rust.vercel.app/no-existe-esta-ruta</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Expected Behavior</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Una pantalla de "no encontrado" propia en español con un camino de vuelta a la app, o redirección a /</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Actual Behavior</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>El body muestra textualmente "Unexpected Application Error!\n404 Not Found" — la pantalla de error por defecto de React Router. Sin header de Biyu, sin link a /register o /login, sin redirección</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Incidence / Severity / Probability of reproduction</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Severidad Media - Una URL mal escrita deja al usuario en una pantalla de error en inglés, sin forma de volver a la app.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>100 % antes de la corrección. No se reproduce desde el 2026-09-28.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Story and Acceptance Criteria affected</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>US-48 · La app pide login. Ningún criterio escrito cubre las rutas inexistentes: se detectó por ataque libre, fuera de los criterios.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Browsers tested</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Google Chrome (Chromium) en Windows 11</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Environment</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Producción https://biyu-rust.vercel.app, navegador Chromium, Windows 11, 2026-09-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="225" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-001
 - Estado: Cerrado · confirmado corregido el 2026-09-28
@@ -3109,7 +3417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -3140,7 +3448,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -3148,103 +3456,124 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Con la categoría activa "Salud" (sembrada), ir a Ajustes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Crear una categoría llamada "salud".</t>
+          <t>2- Tocar el engranaje "Ajustes" arriba a la derecha (en computadora, "Ajustes" en el menú lateral).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Confirmar que en "Categorías" está activa "Salud" (sembrada al crear la cuenta).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- En "Nueva categoría", escribir "salud" (todo en minúsculas) y tocar "Crear categoría".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Mirar la lista de "Categorías" y, en Registrar, la grilla de categorías (escribir un monto y tocar "Siguiente").</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Rechazado con "Ya existe una categoría activa con ese nombre", igual que "Salud".</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Se acepta. Quedan activas "salud" y "Salud".</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Severidad Baja - Quedan dos categorías activas que se ven iguales ("Salud" y "salud") y confunden al registrar.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="B13" s="7" t="inlineStr">
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en la ejecución del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>US-42 · Crear, renombrar y elegir color de categorías. Criterio: "ABM de categorías propias con nombre y color." La regla de no duplicar nombres (CP-CFG-003) compara el texto exacto.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Local: Vite http://localhost:5180 + Supabase local, main 44f1519, Chromium 390×844, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="180" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="24" ht="180" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-019
 - Estado: Abierto · nuevo en la Entrega 1
@@ -3268,7 +3597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -3299,7 +3628,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -3307,110 +3636,124 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Cargar 1250 como tipo de cambio de referencia del mes en Ajustes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Abrir /register, cargar un monto y elegir US$.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>2- Tocar el engranaje "Ajustes" arriba a la derecha (en computadora, "Ajustes" en el menú lateral). En "Tipo de cambio de referencia", elegir el mes actual en "Mes", escribir 1250 en "ARS por USD" y tocar "Guardar tipo de cambio". La lista muestra "$ 1.250,00".</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>3- Mirar el campo "Tipo de cambio (ARS por US$)".</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+          <t>3- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Escribir 100 en el monto y tocar "US$".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Leer el valor precargado en el campo "Tipo de cambio (ARS por US$)" y compararlo con el formato del equivalente "≈ $125.000,00" y con el de Ajustes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>"1.250" o "1.250,00", con el mismo formato que Ajustes y que el equivalente "≈ $125.000,00".</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>"1250.0000".</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Severidad Baja - El valor es correcto, pero se muestra con el formato de la base ("1250.0000") en vez del formato argentino del resto de la app.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en la ejecución del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>US-20 · Sugerir el tipo de cambio de referencia del mes. Criterio: "Si el período tiene TC de referencia, el formulario lo precarga." Se precarga con otro formato.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Local: Vite http://localhost:5180 + Supabase local, main 44f1519, Chromium 390×844, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="165" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="24" ht="165" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-020
 - Estado: Abierto · nuevo en la Entrega 1
@@ -3434,7 +3777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -3465,7 +3808,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -3473,110 +3816,131 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Tener un gasto o ingreso con un monto de 9 o más cifras.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Usar un iPhone con Safari (o un navegador con ancho de pantalla de unos 390 px).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Abrir /dashboard en un celular (ancho ~390 px).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>2- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>3- Mirar la tarjeta "Gastado en…", las tarjetas Ingresos y Balance y la lista "Por categoría".</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+          <t>3- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar". Tocar "Ingreso", escribir 81818491500 en el monto, tocar "Siguiente", en "Cuenta" tocar "Cuenta bancaria" y tocar "Guardar ingreso".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar". Después: escribir 2165003118 en el monto, tocar "Siguiente", tocar el chip "Otros", en "Cuenta" tocar "Efectivo", tocar "Guardar gasto" (aparece "Gasto guardado").</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- En la barra de navegación, tocar "Resumen" (mes actual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Mirar la tarjeta verde "Gastado en …", las tarjetas "Ingresos" y "Balance", y la lista "Por categoría": si algún monto se corta o se sale de su recuadro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Ningún monto se corta ni desborda su contenedor, a cualquier ancho y con montos de hasta el máximo que permite numeric(14,2).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>El total gastado ($2.165.003.118,…) queda cortado por el borde de la tarjeta; Ingresos ($81.818.491.500) y Balance ($79.653.488.381,50) desbordan su casillero; en "Por categoría" el porcentaje "100,0 %" baja de línea.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Severidad Media - El dato principal del Resumen queda ilegible en el celular, sin forma de verlo completo.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>100 % con montos de 9 cifras o más en pantallas de celular.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>US-25 · Total gastado del mes actual al entrar; US-29 · Ingresos y balance del mes ("Muestra total de ingresos y balance = ingresos − gastos"); US-27 · Gasto por categoría en barras. Los montos se muestran pero no se pueden leer.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Safari en iPhone</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Producción (Vercel), Safari en iPhone, ancho ~390 px, 2026-09-29</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="210" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="25" ht="210" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-021
 - Estado: Abierto · reportado el 2026-09-29
@@ -3600,7 +3964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -3631,7 +3995,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -3639,110 +4003,124 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Entrar con una cuenta creada antes de US-68.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Versión donde ocurría: main 7812350, antes de #176. En producción las migraciones de US-68 todavía no estaban aplicadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Observar la pantalla que se abre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>2- Caso A, cuenta anterior a US-68: abrir la app sin sesión y, en /login, entrar con una cuenta creada antes del merge de US-68 (#173). Para reproducirlo en local: crear una cuenta nueva, borrar su fila de configuración (delete from user_setup where user_id = '&lt;id&gt;') y cerrar sesión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>3- Con una cuenta nueva, completar o saltear los 4 pasos del setup con la escritura en user_setup fallando.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Expected Behavior</t>
-        </is>
-      </c>
+          <t>3- Observar la pantalla que se abre después de tocar "Entrar": si va a Registrar o a la configuración inicial ("¿Para qué vas a usar Biyu?").</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Caso B, no se puede guardar el setup: con una cuenta nueva, en la configuración inicial, tocar "Saltear" en "¿Para qué vas a usar Biyu?", "Tus categorías" y "Tus cuentas", y en "Registrá tu primer gasto" tocar "Saltear" al pie. Esto con la escritura en user_setup fallando, como en producción sin la migración, o en local bloqueando las llamadas a /rest/v1/user_setup desde las herramientas de desarrollo (pestaña "Network" → "Block request URL").</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Una cuenta existente entra directo a la app (US-01). Terminar el setup lleva a Registrar y el setup no vuelve a aparecer (US-68).</t>
+          <t>5- Observar si la app avanza a Registrar, si aparece algún mensaje, y qué pasa al tocar "Saltear" otra vez.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Actual Behavior</t>
+          <t>Expected Behavior</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>La cuenta existente es obligada a hacer el setup. Al terminarlo, la app se queda en /setup: el botón vuelve a habilitarse sin ningún mensaje.</t>
+          <t>Una cuenta existente entra directo a la app (US-01). Terminar el setup lleva a Registrar y el setup no vuelve a aparecer (US-68).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>La cuenta existente es obligada a hacer el setup. Al terminarlo, la app se queda en /setup: el botón vuelve a habilitarse sin ningún mensaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Severidad Crítica - Bloquea el acceso a toda la app: los usuarios existentes quedan obligados a hacer el setup, y quien no puede guardarlo queda atrapado en /setup.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>100 % para cuentas anteriores a US-68, y 100 % del bucle mientras falle la escritura en user_setup.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="75" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="18" ht="75" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>US-68 · Configuración inicial al crear la cuenta. Criterio: "Después de crear la cuenta se muestra el setup, y no vuelve a aparecer una vez que se completó o se salteó." También US-01: "Un usuario autenticado que abre la app cae en /register."</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Producción: navegador del usuario. Reproducido y verificado en Chromium y WebKit (Playwright)</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Producción (Vercel + Supabase hosteado), 2026-09-29. Reproducido y verificado en local: Vite http://localhost:5180 + Supabase local, main 7812350</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="390" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="24" ht="390" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-022
 - Estado: Cerrado · corregido en #176 el 2026-09-29; migraciones aplicadas y verificado en producción el 2026-09-29
@@ -3767,7 +4145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -3798,7 +4176,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -3806,103 +4184,124 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Abrir cualquier pantalla de la app.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>1- Versión donde ocurría: producción antes del rediseño de la UI (#161).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Mirar el título de la pestaña y document.documentElement.lang</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="75" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+          <t>2- Abrir https://biyu-rust.vercel.app/login en el navegador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- Leer el título de la pestaña del navegador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Abrir las herramientas de desarrollo (F12), ir a la pestaña "Console", escribir document.documentElement.lang y dar Enter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Repetir los pasos 3 y 4 en /signup, /settings (con sesión iniciada) y en una ruta inexistente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="75" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Título "Biyu" (o por pantalla) y lang="es" (idealmente es-AR, CLAUDE.md fija español rioplatense). NFR-06 pide WCAG 2.1 AA; el criterio 3.1.1 (Idioma de la página) exige que lang coincida con el idioma real, si no los lectores de pantalla leen el español con fonética inglesa</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>document.title = "scaffold" (el nombre del template de Vite), lang = "en" en todas las pantallas probadas</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Severidad Baja - El lector de pantalla lee el español con fonética inglesa y la pestaña dice "scaffold" en vez de Biyu.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="B13" s="7" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>100 % antes de la corrección. No se reproduce desde el 2026-09-28.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Transversal, sin historia propia. NFR-06 (WCAG 2.1 AA), criterio 3.1.1 Idioma de la página: lang tiene que coincidir con el idioma real.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Google Chrome (Chromium) en Windows 11</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Producción https://biyu-rust.vercel.app, /login, /signup, /settings y la ruta 404, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="210" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="24" ht="210" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-002
 - Estado: Cerrado · no se reproduce el 2026-09-28, issue cerrado el 2026-09-29
@@ -3926,7 +4325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -3957,7 +4356,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -3965,103 +4364,117 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Abrir /signup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Versión donde ocurría: producción antes de #141 (US-66 se había perdido en un merge).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Mirar los campos del formulario</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Expected Behavior</t>
-        </is>
-      </c>
+          <t>2- Abrir https://biyu-rust.vercel.app en el navegador, sin sesión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- En la pantalla "Entrar", tocar "Crear una cuenta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>US-66 (02-behavior-spec.md): "quiero confirmar mi contraseña al registrarme escribiéndola dos veces"</t>
+          <t>4- Mirar los campos del formulario "Crear cuenta": qué hay debajo de "Contraseña" y de la lista de criterios, antes del botón "Crear cuenta".</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>US-66 (02-behavior-spec.md): "quiero confirmar mi contraseña al registrarme escribiéndola dos veces"</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Solo aparecen "Email", "Contraseña", la lista de 5 criterios y "Crear cuenta". No hay un segundo campo de confirmación</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Severidad Media - En producción se podía crear una cuenta con una contraseña mal tipeada, que después no se puede reproducir para entrar.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="B13" s="7" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>100 % en producción antes de la corrección. No se reproduce desde el 2026-09-28.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>US-66 · Confirmar contraseña al registrarse. Criterio: "El formulario de /signup tiene un segundo campo 'Confirmar contraseña', con máscara igual que el campo de contraseña."</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Browsers tested</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Google Chrome (Chromium) en Windows 11</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>Browsers tested</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Google Chrome (Chromium) en Windows 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Producción https://biyu-rust.vercel.app/signup, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="240" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="23" ht="240" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-003
 - Estado: Cerrado · no se reproduce el 2026-09-28, issue cerrado el 2026-09-29
@@ -4085,7 +4498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -4124,110 +4537,138 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Con JWT válido, POST /rest/v1/rpc/create_transaction con p_amount: "NaN", p_currency: "ARS", resto de campos válidos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>1- Versión donde ocurría: main antes de #162, contra el stack local (Supabase local y la app en localhost).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Repetir con p_currency: "USD", p_amount: 1, p_fx_rate: "NaN".</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>2- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>3- Abrir /dashboard del período correspondiente.</t>
+          <t>3- Obtener el token de sesión del usuario (en la consola del navegador, con la app abierta: la clave "sb-…-auth-token" de localStorage, campo access_token) y la anon key del proyecto. Las llamadas de los pasos siguientes llevan los encabezados "apikey: &lt;anon key&gt;" y "Authorization: Bearer &lt;token&gt;".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Con ese token, obtener los ids que pide la llamada: GET /rest/v1/categories?select=id,name y GET /rest/v1/accounts?select=id,name,type.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Llamar a POST /rest/v1/rpc/create_transaction con el cuerpo {"p_amount": "NaN", "p_currency": "ARS", "p_category_id": "&lt;id de Otros&gt;", "p_account_id": "&lt;id de Efectivo&gt;", "p_occurred_on": "&lt;fecha de hoy, AAAA-MM-DD&gt;"}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Llamar otra vez con {"p_amount": "1", "p_currency": "USD", "p_fx_rate": "NaN", "p_category_id": "&lt;id de Otros&gt;", "p_account_id": "&lt;id de Efectivo&gt;", "p_occurred_on": "&lt;fecha de hoy&gt;"}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>7- En la app, tocar "Resumen" en la barra de navegación y mirar el mes actual: el total gastado, el balance, "Por categoría" y "Por cuenta".</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Rechazado por I4 (amount &gt; 0) — en Postgres NaN &gt; 0 evalúa true, así que el check no alcanza. upsert_fx_rate ya tiene esta misma protección para fx_rates; create_transaction y el check de debts no.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="105" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="15" ht="105" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Las dos llamadas devuelven un uuid (se crean). En la base: amount: "NaN", amount_ars: "NaN", mismo en ledger_entries. El dashboard muestra "Total gastado $NaN,undefined", "Balance $NaN,undefined", totales por categoría/cuenta "$NaN,undefined" y porcentajes "NaN%". ledger_integrity_violations no lo detecta (en Postgres NaN = NaN es verdadero). Un insert directo a debts con amount: "NaN" también se acepta.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Severidad Crítica - Se guarda un monto que no es un número y el Resumen del mes muestra "$NaN,undefined": se pierde la integridad de los totales (I4).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>100 % antes de la corrección. No se reproduce desde el 2026-09-28.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>US-11 · No se puede guardar monto cero o negativo. Criterio: "La RPC rechaza amount &lt;= 0 aunque el cliente lo deje pasar (I4, C6)."</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright) y llamada directa a la RPC</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Local: http://localhost:5174 + Supabase local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="225" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="26" ht="225" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-004
 - Estado: Cerrado · confirmado corregido el 2026-09-28
@@ -4251,7 +4692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -4282,7 +4723,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -4290,96 +4731,124 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- POST /auth/v1/signup directo (saltando el cliente) con contraseña abc1234 (sin mayúscula ni especial) y por separado con abcd1234 (sin mayúscula ni especial)</t>
+          <t>1- Se reproduce contra Supabase Auth local (política de contraseñas del proyecto local); no se verificó en producción.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2- Obtener la anon key del proyecto local (salida de "supabase status").</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Expected Behavior</t>
-        </is>
-      </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Rechazo — FR-01 exige "validado en cliente **y en el servidor**"; US-67 amplía el criterio a 8+mayúscula+minúscula+número+especial</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Actual Behavior</t>
-        </is>
-      </c>
+          <t>3- Sin pasar por la pantalla de la app, llamar a POST /auth/v1/signup con el encabezado "apikey: &lt;anon key&gt;" y el cuerpo {"email": "&lt;un email nuevo&gt;", "password": "abc1234"}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Repetir la llamada con otro email nuevo y "password": "abcd1234".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Las dos devuelven access_token: cuenta creada con sesión</t>
+          <t>5- Leer las dos respuestas: si traen access_token, la cuenta se creó con sesión.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Rechazo — FR-01 exige "validado en cliente **y en el servidor**"; US-67 amplía el criterio a 8+mayúscula+minúscula+número+especial</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Actual Behavior</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Las dos devuelven access_token: cuenta creada con sesión</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Severidad Media - Una contraseña débil que la pantalla rechaza se puede crear igual yendo directo a la API: la validación queda solo en el cliente (C6).</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>US-67 · Mensaje claro de qué criterio de contraseña falta. Criterio: "El servidor (Supabase Auth) rechaza igual una contraseña que no cumpla (C6)."</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>No aplica: llamada directa a la API de Supabase Auth</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Local: Supabase Auth local (minimum_password_length = 6, password_requirements = ""). No verificado en producción</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="165" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="24" ht="165" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-005
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -4402,7 +4871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -4433,7 +4902,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -4441,110 +4910,131 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Crear un gasto en categoría "Entretenimiento".</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Archivar "Entretenimiento" desde /settings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>2- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar". Después: escribir 8000 en el monto, tocar "Siguiente", tocar el chip "Entretenimiento", tocar "Guardar gasto" (aparece "Gasto guardado").</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>3- Abrir /transactions del período de ese gasto</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+          <t>3- Tocar el engranaje "Ajustes" arriba a la derecha (en computadora, "Ajustes" en el menú lateral).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- En la sección "Categorías", tocar el botón de archivar a la derecha de "Entretenimiento" ("Archivar Entretenimiento"). "Entretenimiento" desaparece de la lista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- En la barra de navegación, tocar "Movimientos" (queda en el mes actual, el del gasto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Buscar el gasto de $8.000 y mirar cómo se muestra su categoría.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>02-behavior-spec.md, sad path "categoría archivada": "Las transacciones históricas la siguen mostrando, **con una marca visual de archivada**" — el dashboard ya lo hace bien, /transactions no</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>El ítem muestra el nombre de la categoría sin ningún indicador de archivada (&lt;span class="truncate"&gt;Entretenimiento&lt;/span&gt;, sin clase ni marca)</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Severidad Baja - En el historial no se distingue una categoría archivada de una activa.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>US-44 · Archivar una categoría sin perder historia. Criterio: "Archivar la saca del formulario; las transacciones históricas la siguen mostrando con marca de archivada."</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="150" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="25" ht="150" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-006
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -4567,7 +5057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -4598,7 +5088,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -4606,110 +5096,131 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Crear un gasto de $50.000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Abrir la app e iniciar sesión: en /login, escribir el email y la contraseña del usuario de prueba y tocar "Entrar". Si aparece la configuración inicial, tocar "Saltear" en sus 4 pasos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Eliminarlo desde /transactions, confirmando el aviso.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+          <t>2- En la barra de navegación de abajo (en computadora, el menú lateral), tocar "Registrar". Después: escribir 50000 en el monto, tocar "Siguiente", tocar el chip "Indumentaria", en "Cuenta" tocar "Efectivo", en "Nota (opcional)" escribir "Campera", tocar "Guardar gasto" (aparece "Gasto guardado").</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>3- Mirar el listado</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+          <t>3- En la barra de navegación, tocar "Movimientos" (mes actual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- En el movimiento "Campera", tocar el tacho ("Eliminar Campera"). Se abre el diálogo "¿Eliminar transacción?".</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>5- Tocar "Eliminar". Aparece "Transacción eliminada".</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>6- Mirar el listado de Movimientos del mes, y después "Últimos movimientos" en el Resumen: si el gasto sigue visible con alguna marca de eliminado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>pre-entrega.md FR-08: "la transacción deja de contarse en los totales pero **permanece visible en el historial con una marca de eliminada**"</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>El ítem desaparece por completo de todos los listados. En la base, deleted_at queda seteado correctamente y el total del mes baja lo esperado</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Severidad Media - Una transacción eliminada desaparece de la vista: el usuario no puede ver qué borró. Los totales sí quedan bien.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="75" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="19" ht="75" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>US-65 · Eliminar una transacción con aviso si toca meses cerrados. Criterio: "El borrado es lógico (deleted_at) y la transacción sale de todos los KPI (I10)." Contradice FR-08: la transacción "permanece visible en el historial con una marca de eliminada".</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="180" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="25" ht="180" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-007
 - Estado: Abierto · se reproduce el 2026-09-28
@@ -4732,7 +5243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.83" customWidth="1" min="1" max="1"/>
@@ -4763,7 +5274,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="45" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Reproduction Steps</t>
@@ -4771,103 +5282,117 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1- Sin sesión, abrir /dashboard?period=2026-06 → redirige a /login?next=%2Fdashboard%3Fperiod%3D2026-06.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+          <t>1- Usar un usuario que ya existe y ya completó o salteó la configuración inicial. Empezar sin sesión: si hay una abierta, ir a Ajustes y tocar "Cerrar sesión".</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>2- Iniciar sesión</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+          <t>2- Escribir en la barra del navegador la dirección de la app seguida de /dashboard?period=2026-06 y dar Enter. La app redirige a /login?next=%2Fdashboard%3Fperiod%3D2026-06.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>3- En "Entrar", escribir el email y la contraseña del usuario y tocar "Entrar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>4- Observar a qué pantalla lleva y la URL final.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Expected Behavior</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Volver a /dashboard?period=2026-06 — AuthForm.tsx sí llama navigate(next), pero algo lo pisa</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Actual Behavior</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Termina siempre en /register, ignorando el next</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Incidence / Severity / Probability of reproduction</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Severidad Media - Quien abre un link directo (por ejemplo al Resumen) sin sesión termina en Registrar después de entrar, no en la pantalla que pidió.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="B13" s="7" t="inlineStr">
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>100 % (se reprodujo en el re-test del 2026-09-28).</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Story and Acceptance Criteria affected</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>US-48 · La app pide login. La historia define que una ruta privada sin sesión redirige a /login?next=&lt;ruta&gt;; el destino de next se ignora al entrar.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Browsers tested</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Chromium (Playwright), emulando un celular de 390×844</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Local, 2026-09-28. Mismo código en producción, probablemente reproduce igual</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="210" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="23" ht="210" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>- Defect ID: DEF-008
 - Estado: Abierto · se reproduce el 2026-09-28

</xml_diff>